<commit_message>
Regenerate pipeline outputs, fast-layer tensors, sandbox curves and HTML reports after the rate-model fix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/irrbb_calc/output/eve_results.xlsx
+++ b/irrbb_calc/output/eve_results.xlsx
@@ -458,13 +458,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-6997548190.8845</v>
+        <v>-6999697446.707</v>
       </c>
       <c r="D2" t="n">
-        <v>-68359595.84784445</v>
+        <v>-68343261.76701321</v>
       </c>
       <c r="E2" t="n">
-        <v>-7065907786.732345</v>
+        <v>-7068040708.474013</v>
       </c>
     </row>
     <row r="3">
@@ -479,13 +479,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1454532238.515</v>
+        <v>1381737612.545</v>
       </c>
       <c r="D3" t="n">
-        <v>219845380.9634366</v>
+        <v>196694663.7578431</v>
       </c>
       <c r="E3" t="n">
-        <v>1674377619.478436</v>
+        <v>1578432276.302843</v>
       </c>
     </row>
     <row r="4">
@@ -521,13 +521,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5913916697.763065</v>
+        <v>5912619717.010962</v>
       </c>
       <c r="D5" t="n">
-        <v>1637121958.72392</v>
+        <v>1481350226.660375</v>
       </c>
       <c r="E5" t="n">
-        <v>7551038656.486984</v>
+        <v>7393969943.671337</v>
       </c>
     </row>
   </sheetData>
@@ -573,13 +573,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>370900745.3935649</v>
+        <v>294659882.8489625</v>
       </c>
       <c r="C2" t="n">
-        <v>1800602293.588707</v>
+        <v>1621696178.4004</v>
       </c>
       <c r="D2" t="n">
-        <v>2171503038.982273</v>
+        <v>1916356061.249362</v>
       </c>
     </row>
   </sheetData>
@@ -658,10 +658,10 @@
         <v>-3083318426.864177</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>-1095.82199864</v>
       </c>
       <c r="F2" t="n">
-        <v>-3083318426.864177</v>
+        <v>-3083319522.686175</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>-3083318426.864177</v>
+        <v>-3083319522.686175</v>
       </c>
     </row>
     <row r="3">
@@ -689,13 +689,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>-2033509970.464682</v>
+        <v>-2035834848.451876</v>
       </c>
       <c r="E3" t="n">
-        <v>-17881642.89649178</v>
+        <v>-17770696.58894503</v>
       </c>
       <c r="F3" t="n">
-        <v>-2051391613.361173</v>
+        <v>-2053605545.040822</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>-2051391613.361173</v>
+        <v>-2053605545.040822</v>
       </c>
     </row>
     <row r="4">
@@ -723,13 +723,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-1668798765.669185</v>
+        <v>-1668639400.472654</v>
       </c>
       <c r="E4" t="n">
-        <v>-79484758.04393794</v>
+        <v>-79580111.73322277</v>
       </c>
       <c r="F4" t="n">
-        <v>-1748283523.713123</v>
+        <v>-1748219512.205877</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>-1748283523.713123</v>
+        <v>-1748219512.205877</v>
       </c>
     </row>
     <row r="5">
@@ -757,13 +757,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1458552649.995376</v>
+        <v>1383975066.680009</v>
       </c>
       <c r="E5" t="n">
-        <v>214501871.3609806</v>
+        <v>198487045.1890026</v>
       </c>
       <c r="F5" t="n">
-        <v>1673054521.356357</v>
+        <v>1582462111.869012</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -771,7 +771,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1673054521.356357</v>
+        <v>1582462111.869012</v>
       </c>
     </row>
     <row r="6">
@@ -791,13 +791,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>-88122071.84726256</v>
+        <v>-84725905.57052767</v>
       </c>
       <c r="E6" t="n">
-        <v>-7833877.715764532</v>
+        <v>-15687823.29937529</v>
       </c>
       <c r="F6" t="n">
-        <v>-95955949.56302708</v>
+        <v>-100413728.869903</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>-95955949.56302708</v>
+        <v>-100413728.869903</v>
       </c>
     </row>
     <row r="7">
@@ -893,13 +893,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1570971611.957587</v>
+        <v>1571001211.012396</v>
       </c>
       <c r="E9" t="n">
-        <v>428848751.7512775</v>
+        <v>404327489.4139838</v>
       </c>
       <c r="F9" t="n">
-        <v>1999820363.708864</v>
+        <v>1975328700.42638</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1999820363.708864</v>
+        <v>1975328700.42638</v>
       </c>
     </row>
     <row r="10">
@@ -927,13 +927,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3906360955.621425</v>
+        <v>3906042905.721296</v>
       </c>
       <c r="E10" t="n">
-        <v>1458278927.469274</v>
+        <v>1332764827.755641</v>
       </c>
       <c r="F10" t="n">
-        <v>5364639883.090699</v>
+        <v>5238807733.476937</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>5364639883.090699</v>
+        <v>5238807733.476937</v>
       </c>
     </row>
     <row r="11">
@@ -964,10 +964,10 @@
         <v>-3399019507.228214</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>-1021.200000000632</v>
       </c>
       <c r="F11" t="n">
-        <v>-3399019507.228214</v>
+        <v>-3399020528.428214</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>-3399019507.228214</v>
+        <v>-3399020528.428214</v>
       </c>
     </row>
     <row r="12">
@@ -995,13 +995,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>-2059896778.52325</v>
+        <v>-2062061957.591353</v>
       </c>
       <c r="E12" t="n">
-        <v>-18189076.41122006</v>
+        <v>-18075806.41501321</v>
       </c>
       <c r="F12" t="n">
-        <v>-2078085854.93447</v>
+        <v>-2080137764.006366</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>-2078085854.93447</v>
+        <v>-2080137764.006366</v>
       </c>
     </row>
     <row r="13">
@@ -1029,13 +1029,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>-1769546823.174845</v>
+        <v>-1769514049.559464</v>
       </c>
       <c r="E13" t="n">
-        <v>-19491678.54685305</v>
+        <v>-19587863.29355559</v>
       </c>
       <c r="F13" t="n">
-        <v>-1789038501.721698</v>
+        <v>-1789101912.853019</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>-1789038501.721698</v>
+        <v>-1789101912.853019</v>
       </c>
     </row>
     <row r="14">
@@ -1063,13 +1063,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1643124559.975856</v>
+        <v>1567816110.294005</v>
       </c>
       <c r="E14" t="n">
-        <v>233986076.6765736</v>
+        <v>217729727.858979</v>
       </c>
       <c r="F14" t="n">
-        <v>1877110636.652429</v>
+        <v>1785545838.152984</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1877110636.652429</v>
+        <v>1785545838.152984</v>
       </c>
     </row>
     <row r="15">
@@ -1097,13 +1097,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>-97232772.38659269</v>
+        <v>-96176198.51548576</v>
       </c>
       <c r="E15" t="n">
-        <v>35066.31536514341</v>
+        <v>-6011170.003274525</v>
       </c>
       <c r="F15" t="n">
-        <v>-97197706.07122755</v>
+        <v>-102187368.5187603</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>-97197706.07122755</v>
+        <v>-102187368.5187603</v>
       </c>
     </row>
     <row r="16">
@@ -1199,13 +1199,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1798515365.395193</v>
+        <v>1797338581.993386</v>
       </c>
       <c r="E18" t="n">
-        <v>474190931.7426074</v>
+        <v>446737695.5933225</v>
       </c>
       <c r="F18" t="n">
-        <v>2272706297.1378</v>
+        <v>2244076277.586709</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>2272706297.1378</v>
+        <v>2244076277.586709</v>
       </c>
     </row>
     <row r="19">
@@ -1233,13 +1233,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4607700448.758251</v>
+        <v>4606443436.747486</v>
       </c>
       <c r="E19" t="n">
-        <v>875882286.067891</v>
+        <v>741421019.612464</v>
       </c>
       <c r="F19" t="n">
-        <v>5483582734.826142</v>
+        <v>5347864456.35995</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>5483582734.826142</v>
+        <v>5347864456.35995</v>
       </c>
     </row>
     <row r="20">
@@ -1270,10 +1270,10 @@
         <v>-3163578369.50797</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>-1095.96497184</v>
       </c>
       <c r="F20" t="n">
-        <v>-3163578369.50797</v>
+        <v>-3163579465.472941</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>-3163578369.50797</v>
+        <v>-3163579465.472941</v>
       </c>
     </row>
     <row r="21">
@@ -1301,13 +1301,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>-2053193093.438182</v>
+        <v>-2055406273.158957</v>
       </c>
       <c r="E21" t="n">
-        <v>-18104332.50265941</v>
+        <v>-17991696.55184771</v>
       </c>
       <c r="F21" t="n">
-        <v>-2071297425.940841</v>
+        <v>-2073397969.710804</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>-2071297425.940841</v>
+        <v>-2073397969.710804</v>
       </c>
     </row>
     <row r="22">
@@ -1335,13 +1335,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>-1702309538.160335</v>
+        <v>-1702263538.499749</v>
       </c>
       <c r="E22" t="n">
-        <v>-59770203.50213085</v>
+        <v>-59866302.32310096</v>
       </c>
       <c r="F22" t="n">
-        <v>-1762079741.662466</v>
+        <v>-1762129840.82285</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>-1762079741.662466</v>
+        <v>-1762129840.82285</v>
       </c>
     </row>
     <row r="23">
@@ -1369,13 +1369,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1507748153.824305</v>
+        <v>1430611516.190344</v>
       </c>
       <c r="E23" t="n">
-        <v>220719797.2200679</v>
+        <v>204410595.5587594</v>
       </c>
       <c r="F23" t="n">
-        <v>1728467951.044373</v>
+        <v>1635022111.749104</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>1728467951.044373</v>
+        <v>1635022111.749104</v>
       </c>
     </row>
     <row r="24">
@@ -1403,13 +1403,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>-91937498.61060362</v>
+        <v>-88146220.94866616</v>
       </c>
       <c r="E24" t="n">
-        <v>-4883575.035104213</v>
+        <v>-13245378.91382747</v>
       </c>
       <c r="F24" t="n">
-        <v>-96821073.64570779</v>
+        <v>-101391599.8624936</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>-96821073.64570779</v>
+        <v>-101391599.8624936</v>
       </c>
     </row>
     <row r="25">
@@ -1505,13 +1505,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1630471775.3176</v>
+        <v>1630303405.995301</v>
       </c>
       <c r="E27" t="n">
-        <v>442250387.2924819</v>
+        <v>416903410.0818864</v>
       </c>
       <c r="F27" t="n">
-        <v>2072722162.610082</v>
+        <v>2047206816.077187</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>2072722162.610082</v>
+        <v>2047206816.077187</v>
       </c>
     </row>
     <row r="28">
@@ -1539,13 +1539,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>4077199274.881555</v>
+        <v>4076747099.872595</v>
       </c>
       <c r="E28" t="n">
-        <v>1343700122.427795</v>
+        <v>1214999554.923893</v>
       </c>
       <c r="F28" t="n">
-        <v>5420899397.30935</v>
+        <v>5291746654.796488</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>5420899397.30935</v>
+        <v>5291746654.796488</v>
       </c>
     </row>
     <row r="29">
@@ -1576,10 +1576,10 @@
         <v>-3290858979.57491</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>-1095.81332928</v>
       </c>
       <c r="F29" t="n">
-        <v>-3290858979.57491</v>
+        <v>-3290860075.38824</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1587,7 +1587,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>-3290858979.57491</v>
+        <v>-3290860075.38824</v>
       </c>
     </row>
     <row r="30">
@@ -1607,13 +1607,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>-2037818484.095129</v>
+        <v>-2040109369.00206</v>
       </c>
       <c r="E30" t="n">
-        <v>-17938869.19535578</v>
+        <v>-17827496.49511871</v>
       </c>
       <c r="F30" t="n">
-        <v>-2055757353.290485</v>
+        <v>-2057936865.497179</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>-2055757353.290485</v>
+        <v>-2057936865.497179</v>
       </c>
     </row>
     <row r="31">
@@ -1641,13 +1641,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>-1728145584.153817</v>
+        <v>-1727986719.141655</v>
       </c>
       <c r="E31" t="n">
-        <v>-43895094.04253259</v>
+        <v>-43990450.20683838</v>
       </c>
       <c r="F31" t="n">
-        <v>-1772040678.196349</v>
+        <v>-1771977169.348494</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>-1772040678.196349</v>
+        <v>-1771977169.348494</v>
       </c>
     </row>
     <row r="32">
@@ -1675,13 +1675,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1578701859.574636</v>
+        <v>1505976976.942232</v>
       </c>
       <c r="E32" t="n">
-        <v>226203822.4080096</v>
+        <v>210260783.4968137</v>
       </c>
       <c r="F32" t="n">
-        <v>1804905681.982645</v>
+        <v>1716237760.439046</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>1804905681.982645</v>
+        <v>1716237760.439046</v>
       </c>
     </row>
     <row r="33">
@@ -1709,13 +1709,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>-92559919.51819681</v>
+        <v>-91746843.35194483</v>
       </c>
       <c r="E33" t="n">
-        <v>-3663743.394470075</v>
+        <v>-9319613.642388146</v>
       </c>
       <c r="F33" t="n">
-        <v>-96223662.91266692</v>
+        <v>-101066456.9943329</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>-96223662.91266692</v>
+        <v>-101066456.9943329</v>
       </c>
     </row>
     <row r="34">
@@ -1811,13 +1811,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1718919941.512958</v>
+        <v>1718070353.025799</v>
       </c>
       <c r="E36" t="n">
-        <v>456993116.105382</v>
+        <v>430613497.4205008</v>
       </c>
       <c r="F36" t="n">
-        <v>2175913057.61834</v>
+        <v>2148683850.4463</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>2175913057.61834</v>
+        <v>2148683850.4463</v>
       </c>
     </row>
     <row r="37">
@@ -1845,13 +1845,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4368931624.263527</v>
+        <v>4367865837.054114</v>
       </c>
       <c r="E37" t="n">
-        <v>1046434276.270612</v>
+        <v>915899295.0771817</v>
       </c>
       <c r="F37" t="n">
-        <v>5415365900.53414</v>
+        <v>5283765132.131296</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>5415365900.53414</v>
+        <v>5283765132.131296</v>
       </c>
     </row>
     <row r="38">
@@ -1882,10 +1882,10 @@
         <v>-3220163562.207465</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>-1095.79228608</v>
       </c>
       <c r="F38" t="n">
-        <v>-3220163562.207465</v>
+        <v>-3220164657.999752</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>-3220163562.207465</v>
+        <v>-3220164657.999752</v>
       </c>
     </row>
     <row r="39">
@@ -1913,13 +1913,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>-2033512180.224723</v>
+        <v>-2035829947.451668</v>
       </c>
       <c r="E39" t="n">
-        <v>-17887960.24661228</v>
+        <v>-17776971.56842878</v>
       </c>
       <c r="F39" t="n">
-        <v>-2051400140.471335</v>
+        <v>-2053606919.020097</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>-2051400140.471335</v>
+        <v>-2053606919.020097</v>
       </c>
     </row>
     <row r="40">
@@ -1947,13 +1947,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>-1706745091.041668</v>
+        <v>-1706567718.532032</v>
       </c>
       <c r="E40" t="n">
-        <v>-56666566.04319399</v>
+        <v>-56761800.53062917</v>
       </c>
       <c r="F40" t="n">
-        <v>-1763411657.084862</v>
+        <v>-1763329519.062661</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>-1763411657.084862</v>
+        <v>-1763329519.062661</v>
       </c>
     </row>
     <row r="41">
@@ -1981,13 +1981,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1537787790.523137</v>
+        <v>1464911848.915145</v>
       </c>
       <c r="E41" t="n">
-        <v>222024365.280676</v>
+        <v>206105624.0048289</v>
       </c>
       <c r="F41" t="n">
-        <v>1759812155.803813</v>
+        <v>1671017472.919974</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1759812155.803813</v>
+        <v>1671017472.919974</v>
       </c>
     </row>
     <row r="42">
@@ -2015,13 +2015,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>-90709178.87877671</v>
+        <v>-89260975.01371798</v>
       </c>
       <c r="E42" t="n">
-        <v>-5305093.713434674</v>
+        <v>-11477510.98777739</v>
       </c>
       <c r="F42" t="n">
-        <v>-96014272.59221135</v>
+        <v>-100738486.0014953</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>-96014272.59221135</v>
+        <v>-100738486.0014953</v>
       </c>
     </row>
     <row r="43">
@@ -2117,13 +2117,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1668202615.968628</v>
+        <v>1667639460.942172</v>
       </c>
       <c r="E45" t="n">
-        <v>447109589.1876891</v>
+        <v>421374669.2835167</v>
       </c>
       <c r="F45" t="n">
-        <v>2115312205.156318</v>
+        <v>2089014130.225689</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>2115312205.156318</v>
+        <v>2089014130.225689</v>
       </c>
     </row>
     <row r="46">
@@ -2151,13 +2151,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4210551146.545216</v>
+        <v>4209706772.111761</v>
       </c>
       <c r="E46" t="n">
-        <v>1181295358.420205</v>
+        <v>1052638446.31821</v>
       </c>
       <c r="F46" t="n">
-        <v>5391846504.965421</v>
+        <v>5262345218.429971</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>5391846504.965421</v>
+        <v>5262345218.429971</v>
       </c>
     </row>
     <row r="47">
@@ -2219,13 +2219,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>-2059886322.574671</v>
+        <v>-2062058668.263331</v>
       </c>
       <c r="E48" t="n">
-        <v>-18182583.66750258</v>
+        <v>-18069356.33798468</v>
       </c>
       <c r="F48" t="n">
-        <v>-2078068906.242174</v>
+        <v>-2080128024.601315</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>-2078068906.242174</v>
+        <v>-2080128024.601315</v>
       </c>
     </row>
     <row r="49">
@@ -2253,13 +2253,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>-1728919520.482759</v>
+        <v>-1728904985.836331</v>
       </c>
       <c r="E49" t="n">
-        <v>-43915720.07691476</v>
+        <v>-44012024.86888601</v>
       </c>
       <c r="F49" t="n">
-        <v>-1772835240.559674</v>
+        <v>-1772917010.705217</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>-1772835240.559674</v>
+        <v>-1772917010.705217</v>
       </c>
     </row>
     <row r="50">
@@ -2287,13 +2287,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1556339566.542586</v>
+        <v>1479015826.853442</v>
       </c>
       <c r="E50" t="n">
-        <v>225855044.9934797</v>
+        <v>209484658.562648</v>
       </c>
       <c r="F50" t="n">
-        <v>1782194611.536066</v>
+        <v>1688500485.41609</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>1782194611.536066</v>
+        <v>1688500485.41609</v>
       </c>
     </row>
     <row r="51">
@@ -2321,13 +2321,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>-94296466.56902525</v>
+        <v>-91152904.78500237</v>
       </c>
       <c r="E51" t="n">
-        <v>-2842104.74285167</v>
+        <v>-10701706.44809381</v>
       </c>
       <c r="F51" t="n">
-        <v>-97138571.31187685</v>
+        <v>-101854611.2330962</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2335,7 +2335,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>-97138571.31187685</v>
+        <v>-101854611.2330962</v>
       </c>
     </row>
     <row r="52">
@@ -2423,13 +2423,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1690030152.036259</v>
+        <v>1689551241.756139</v>
       </c>
       <c r="E54" t="n">
-        <v>454163894.2464075</v>
+        <v>428046921.0083535</v>
       </c>
       <c r="F54" t="n">
-        <v>2144194046.282666</v>
+        <v>2117598162.764492</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>2144194046.282666</v>
+        <v>2117598162.764492</v>
       </c>
     </row>
     <row r="55">
@@ -2457,13 +2457,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>4259378078.146482</v>
+        <v>4258672231.387065</v>
       </c>
       <c r="E55" t="n">
-        <v>1191921704.471508</v>
+        <v>1060871481.666171</v>
       </c>
       <c r="F55" t="n">
-        <v>5451299782.61799</v>
+        <v>5319543713.053237</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2471,7 +2471,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>5451299782.61799</v>
+        <v>5319543713.053237</v>
       </c>
     </row>
     <row r="56">
@@ -2494,10 +2494,10 @@
         <v>-3297443579.731035</v>
       </c>
       <c r="E56" t="n">
-        <v>0</v>
+        <v>-1095.92701736</v>
       </c>
       <c r="F56" t="n">
-        <v>-3297443579.731035</v>
+        <v>-3297444675.658052</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>-3297443579.731035</v>
+        <v>-3297444675.658052</v>
       </c>
     </row>
     <row r="57">
@@ -2525,13 +2525,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>-2051933627.528429</v>
+        <v>-2054147066.18232</v>
       </c>
       <c r="E57" t="n">
-        <v>-18096231.0347071</v>
+        <v>-17983662.59355108</v>
       </c>
       <c r="F57" t="n">
-        <v>-2070029858.563136</v>
+        <v>-2072130728.775872</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>-2070029858.563136</v>
+        <v>-2072130728.775872</v>
       </c>
     </row>
     <row r="58">
@@ -2559,13 +2559,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>-1738141500.890211</v>
+        <v>-1738070634.351016</v>
       </c>
       <c r="E58" t="n">
-        <v>-38197525.93889388</v>
+        <v>-38293460.94437269</v>
       </c>
       <c r="F58" t="n">
-        <v>-1776339026.829105</v>
+        <v>-1776364095.295389</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>-1776339026.829105</v>
+        <v>-1776364095.295389</v>
       </c>
     </row>
     <row r="59">
@@ -2593,13 +2593,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1584506641.909419</v>
+        <v>1509299454.73327</v>
       </c>
       <c r="E59" t="n">
-        <v>227874324.5332424</v>
+        <v>211683870.2150885</v>
       </c>
       <c r="F59" t="n">
-        <v>1812380966.442661</v>
+        <v>1720983324.948359</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>1812380966.442661</v>
+        <v>1720983324.948359</v>
       </c>
     </row>
     <row r="60">
@@ -2627,13 +2627,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>-94337969.37071514</v>
+        <v>-92528512.11000258</v>
       </c>
       <c r="E60" t="n">
-        <v>-2484673.816937748</v>
+        <v>-9119557.675629426</v>
       </c>
       <c r="F60" t="n">
-        <v>-96822643.18765292</v>
+        <v>-101648069.785632</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2641,7 +2641,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>-96822643.18765292</v>
+        <v>-101648069.785632</v>
       </c>
     </row>
     <row r="61">
@@ -2729,13 +2729,13 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1725405580.252823</v>
+        <v>1724635591.07882</v>
       </c>
       <c r="E63" t="n">
-        <v>459821733.4067891</v>
+        <v>433301083.4391299</v>
       </c>
       <c r="F63" t="n">
-        <v>2185227313.659612</v>
+        <v>2157936674.51795</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2743,7 +2743,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>2185227313.659612</v>
+        <v>2157936674.51795</v>
       </c>
     </row>
     <row r="64">
@@ -2763,13 +2763,13 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>4378271708.326949</v>
+        <v>4377306022.247397</v>
       </c>
       <c r="E64" t="n">
-        <v>1067313875.381661</v>
+        <v>935656590.6933227</v>
       </c>
       <c r="F64" t="n">
-        <v>5445585583.70861</v>
+        <v>5312962612.94072</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2777,7 +2777,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>5445585583.70861</v>
+        <v>5312962612.94072</v>
       </c>
     </row>
   </sheetData>
@@ -2848,13 +2848,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>62135982.72908232</v>
+        <v>-11499397.94553286</v>
       </c>
       <c r="C2" t="n">
-        <v>1979622874.554037</v>
+        <v>1805733237.543785</v>
       </c>
       <c r="D2" t="n">
-        <v>2041758857.283119</v>
+        <v>1794233839.598252</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -2862,16 +2862,16 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-129744181.6991534</v>
+        <v>-122122221.6511104</v>
       </c>
       <c r="G2" t="n">
-        <v>-10.81201514159612</v>
+        <v>-10.1768518042592</v>
       </c>
       <c r="H2" t="n">
-        <v>-129744181.6991534</v>
+        <v>-122122221.6511104</v>
       </c>
       <c r="I2" t="n">
-        <v>-10.81201514159612</v>
+        <v>-10.1768518042592</v>
       </c>
     </row>
     <row r="3">
@@ -2881,13 +2881,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>723644492.8163977</v>
+        <v>644826416.1403605</v>
       </c>
       <c r="C3" t="n">
-        <v>1589267517.854559</v>
+        <v>1405066494.163117</v>
       </c>
       <c r="D3" t="n">
-        <v>2312912010.670957</v>
+        <v>2049892910.303477</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -2895,16 +2895,16 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>141408971.688684</v>
+        <v>133536849.0541148</v>
       </c>
       <c r="G3" t="n">
-        <v>11.784080974057</v>
+        <v>11.12807075450957</v>
       </c>
       <c r="H3" t="n">
-        <v>70704485.84434199</v>
+        <v>66768424.52705741</v>
       </c>
       <c r="I3" t="n">
-        <v>5.892040487028499</v>
+        <v>5.564035377254784</v>
       </c>
     </row>
     <row r="4">
@@ -2914,13 +2914,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>204400704.3063711</v>
+        <v>128267619.9428985</v>
       </c>
       <c r="C4" t="n">
-        <v>1920694592.536643</v>
+        <v>1741991483.446984</v>
       </c>
       <c r="D4" t="n">
-        <v>2125095296.843014</v>
+        <v>1870259103.389882</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -2928,16 +2928,16 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-46407742.13925838</v>
+        <v>-46096957.85948014</v>
       </c>
       <c r="G4" t="n">
-        <v>-3.867311844938199</v>
+        <v>-3.841413154956678</v>
       </c>
       <c r="H4" t="n">
-        <v>-46407742.13925838</v>
+        <v>-46096957.85948014</v>
       </c>
       <c r="I4" t="n">
-        <v>-3.867311844938199</v>
+        <v>-3.841413154956678</v>
       </c>
     </row>
     <row r="5">
@@ -2947,13 +2947,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>517170458.0090675</v>
+        <v>441211255.9515758</v>
       </c>
       <c r="C5" t="n">
-        <v>1688889491.82272</v>
+        <v>1510390903.507896</v>
       </c>
       <c r="D5" t="n">
-        <v>2206059949.831788</v>
+        <v>1951602159.459472</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -2961,16 +2961,16 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>34556910.84951544</v>
+        <v>35246098.21010947</v>
       </c>
       <c r="G5" t="n">
-        <v>2.879742570792953</v>
+        <v>2.937174850842456</v>
       </c>
       <c r="H5" t="n">
-        <v>17278455.42475772</v>
+        <v>17623049.10505474</v>
       </c>
       <c r="I5" t="n">
-        <v>1.439871285396477</v>
+        <v>1.468587425421228</v>
       </c>
     </row>
     <row r="6">
@@ -2980,13 +2980,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>365411540.6843474</v>
+        <v>290435878.7641941</v>
       </c>
       <c r="C6" t="n">
-        <v>1781891035.661898</v>
+        <v>1605422703.504003</v>
       </c>
       <c r="D6" t="n">
-        <v>2147302576.346245</v>
+        <v>1895858582.268197</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -2994,16 +2994,16 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>-24200462.63602734</v>
+        <v>-20497478.98116589</v>
       </c>
       <c r="G6" t="n">
-        <v>-2.016705219668945</v>
+        <v>-1.70812324843049</v>
       </c>
       <c r="H6" t="n">
-        <v>-24200462.63602734</v>
+        <v>-20497478.98116589</v>
       </c>
       <c r="I6" t="n">
-        <v>-2.016705219668945</v>
+        <v>-1.70812324843049</v>
       </c>
     </row>
     <row r="7">
@@ -3013,13 +3013,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>376451700.0145519</v>
+        <v>298928954.0276618</v>
       </c>
       <c r="C7" t="n">
-        <v>1819674659.937271</v>
+        <v>1638294398.295353</v>
       </c>
       <c r="D7" t="n">
-        <v>2196126359.951823</v>
+        <v>1937223352.323015</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -3027,16 +3027,16 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>24623320.96955013</v>
+        <v>20867291.07365227</v>
       </c>
       <c r="G7" t="n">
-        <v>2.051943414129178</v>
+        <v>1.738940922804356</v>
       </c>
       <c r="H7" t="n">
-        <v>12311660.48477507</v>
+        <v>10433645.53682613</v>
       </c>
       <c r="I7" t="n">
-        <v>1.025971707064589</v>
+        <v>0.8694704614021779</v>
       </c>
     </row>
     <row r="8">
@@ -3046,13 +3046,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>506327252.9688012</v>
+        <v>429051275.6851131</v>
       </c>
       <c r="C8" t="n">
-        <v>1720315670.913024</v>
+        <v>1539327935.588841</v>
       </c>
       <c r="D8" t="n">
-        <v>2226642923.881825</v>
+        <v>1968379211.273955</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -3060,16 +3060,16 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>55139884.89955282</v>
+        <v>52023150.02459216</v>
       </c>
       <c r="G8" t="n">
-        <v>4.594990408296069</v>
+        <v>4.335262502049346</v>
       </c>
       <c r="H8" t="n">
-        <v>27569942.44977641</v>
+        <v>26011575.01229608</v>
       </c>
       <c r="I8" t="n">
-        <v>2.297495204148035</v>
+        <v>2.167631251024673</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regenerate pipeline outputs, fast-layer tensors (incl. FTP), sandbox curves, HTML reports and ALM charts on a fresh balance-sheet draw
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/irrbb_calc/output/eve_results.xlsx
+++ b/irrbb_calc/output/eve_results.xlsx
@@ -458,13 +458,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-6999697446.707</v>
+        <v>-7029875728.557</v>
       </c>
       <c r="D2" t="n">
-        <v>-68343261.76701321</v>
+        <v>-68876490.58171675</v>
       </c>
       <c r="E2" t="n">
-        <v>-7068040708.474013</v>
+        <v>-7098752219.138717</v>
       </c>
     </row>
     <row r="3">
@@ -479,13 +479,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1381737612.545</v>
+        <v>1448593436.95</v>
       </c>
       <c r="D3" t="n">
-        <v>196694663.7578431</v>
+        <v>220854444.8128947</v>
       </c>
       <c r="E3" t="n">
-        <v>1578432276.302843</v>
+        <v>1669447881.762895</v>
       </c>
     </row>
     <row r="4">
@@ -521,13 +521,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5912619717.010962</v>
+        <v>5915661236.118138</v>
       </c>
       <c r="D5" t="n">
-        <v>1481350226.660375</v>
+        <v>1476394748.315891</v>
       </c>
       <c r="E5" t="n">
-        <v>7393969943.671337</v>
+        <v>7392055984.43403</v>
       </c>
     </row>
   </sheetData>
@@ -573,13 +573,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>294659882.8489625</v>
+        <v>334378944.5111387</v>
       </c>
       <c r="C2" t="n">
-        <v>1621696178.4004</v>
+        <v>1640367252.296265</v>
       </c>
       <c r="D2" t="n">
-        <v>1916356061.249362</v>
+        <v>1974746196.807404</v>
       </c>
     </row>
   </sheetData>
@@ -689,13 +689,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>-2035834848.451876</v>
+        <v>-2065268842.228333</v>
       </c>
       <c r="E3" t="n">
-        <v>-17770696.58894503</v>
+        <v>-18503037.99657344</v>
       </c>
       <c r="F3" t="n">
-        <v>-2053605545.040822</v>
+        <v>-2083771880.224906</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>-2053605545.040822</v>
+        <v>-2083771880.224906</v>
       </c>
     </row>
     <row r="4">
@@ -723,13 +723,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-1668639400.472654</v>
+        <v>-1668980907.697917</v>
       </c>
       <c r="E4" t="n">
-        <v>-79580111.73322277</v>
+        <v>-79375404.67044692</v>
       </c>
       <c r="F4" t="n">
-        <v>-1748219512.205877</v>
+        <v>-1748356312.368364</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>-1748219512.205877</v>
+        <v>-1748356312.368364</v>
       </c>
     </row>
     <row r="5">
@@ -757,13 +757,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1383975066.680009</v>
+        <v>1468406371.257062</v>
       </c>
       <c r="E5" t="n">
-        <v>198487045.1890026</v>
+        <v>206250744.6600633</v>
       </c>
       <c r="F5" t="n">
-        <v>1582462111.869012</v>
+        <v>1674657115.917126</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -771,7 +771,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1582462111.869012</v>
+        <v>1674657115.917126</v>
       </c>
     </row>
     <row r="6">
@@ -791,13 +791,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>-84725905.57052767</v>
+        <v>-107033748.660902</v>
       </c>
       <c r="E6" t="n">
-        <v>-15687823.29937529</v>
+        <v>9845891.559621761</v>
       </c>
       <c r="F6" t="n">
-        <v>-100413728.869903</v>
+        <v>-97187857.10128027</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>-100413728.869903</v>
+        <v>-97187857.10128027</v>
       </c>
     </row>
     <row r="7">
@@ -893,13 +893,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1571001211.012396</v>
+        <v>1571750373.523791</v>
       </c>
       <c r="E9" t="n">
-        <v>404327489.4139838</v>
+        <v>400717773.0341281</v>
       </c>
       <c r="F9" t="n">
-        <v>1975328700.42638</v>
+        <v>1972468146.557919</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1975328700.42638</v>
+        <v>1972468146.557919</v>
       </c>
     </row>
     <row r="10">
@@ -927,13 +927,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3906042905.721296</v>
+        <v>3908964962.211827</v>
       </c>
       <c r="E10" t="n">
-        <v>1332764827.755641</v>
+        <v>1330976793.464843</v>
       </c>
       <c r="F10" t="n">
-        <v>5238807733.476937</v>
+        <v>5239941755.67667</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>5238807733.476937</v>
+        <v>5239941755.67667</v>
       </c>
     </row>
     <row r="11">
@@ -995,13 +995,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>-2062061957.591353</v>
+        <v>-2092577080.256001</v>
       </c>
       <c r="E12" t="n">
-        <v>-18075806.41501321</v>
+        <v>-18820582.57208558</v>
       </c>
       <c r="F12" t="n">
-        <v>-2080137764.006366</v>
+        <v>-2111397662.828087</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>-2080137764.006366</v>
+        <v>-2111397662.828087</v>
       </c>
     </row>
     <row r="13">
@@ -1029,13 +1029,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>-1769514049.559464</v>
+        <v>-1769584180.096029</v>
       </c>
       <c r="E13" t="n">
-        <v>-19587863.29355559</v>
+        <v>-19381966.56324614</v>
       </c>
       <c r="F13" t="n">
-        <v>-1789101912.853019</v>
+        <v>-1788966146.659275</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>-1789101912.853019</v>
+        <v>-1788966146.659275</v>
       </c>
     </row>
     <row r="14">
@@ -1063,13 +1063,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1567816110.294005</v>
+        <v>1645505324.592738</v>
       </c>
       <c r="E14" t="n">
-        <v>217729727.858979</v>
+        <v>224711995.9439799</v>
       </c>
       <c r="F14" t="n">
-        <v>1785545838.152984</v>
+        <v>1870217320.536718</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1785545838.152984</v>
+        <v>1870217320.536718</v>
       </c>
     </row>
     <row r="15">
@@ -1097,13 +1097,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>-96176198.51548576</v>
+        <v>-101858202.2109235</v>
       </c>
       <c r="E15" t="n">
-        <v>-6011170.003274525</v>
+        <v>870299.6453202302</v>
       </c>
       <c r="F15" t="n">
-        <v>-102187368.5187603</v>
+        <v>-100987902.5656033</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>-102187368.5187603</v>
+        <v>-100987902.5656033</v>
       </c>
     </row>
     <row r="16">
@@ -1199,13 +1199,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1797338581.993386</v>
+        <v>1798790146.735549</v>
       </c>
       <c r="E18" t="n">
-        <v>446737695.5933225</v>
+        <v>442809147.9247949</v>
       </c>
       <c r="F18" t="n">
-        <v>2244076277.586709</v>
+        <v>2241599294.660344</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>2244076277.586709</v>
+        <v>2241599294.660344</v>
       </c>
     </row>
     <row r="19">
@@ -1233,13 +1233,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4606443436.747486</v>
+        <v>4607298938.211198</v>
       </c>
       <c r="E19" t="n">
-        <v>741421019.612464</v>
+        <v>740965577.77644</v>
       </c>
       <c r="F19" t="n">
-        <v>5347864456.35995</v>
+        <v>5348264515.987638</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>5347864456.35995</v>
+        <v>5348264515.987638</v>
       </c>
     </row>
     <row r="20">
@@ -1301,13 +1301,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>-2055406273.158957</v>
+        <v>-2085649134.717873</v>
       </c>
       <c r="E21" t="n">
-        <v>-17991696.55184771</v>
+        <v>-18733127.49967238</v>
       </c>
       <c r="F21" t="n">
-        <v>-2073397969.710804</v>
+        <v>-2104382262.217545</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>-2073397969.710804</v>
+        <v>-2104382262.217545</v>
       </c>
     </row>
     <row r="22">
@@ -1335,13 +1335,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>-1702263538.499749</v>
+        <v>-1702361985.445435</v>
       </c>
       <c r="E22" t="n">
-        <v>-59866302.32310096</v>
+        <v>-59660528.0241149</v>
       </c>
       <c r="F22" t="n">
-        <v>-1762129840.82285</v>
+        <v>-1762022513.469549</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>-1762129840.82285</v>
+        <v>-1762022513.469549</v>
       </c>
     </row>
     <row r="23">
@@ -1369,13 +1369,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1430611516.190344</v>
+        <v>1515960029.562124</v>
       </c>
       <c r="E23" t="n">
-        <v>204410595.5587594</v>
+        <v>212130771.4154197</v>
       </c>
       <c r="F23" t="n">
-        <v>1635022111.749104</v>
+        <v>1728090800.977544</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>1635022111.749104</v>
+        <v>1728090800.977544</v>
       </c>
     </row>
     <row r="24">
@@ -1403,13 +1403,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>-88146220.94866616</v>
+        <v>-107743033.3319404</v>
       </c>
       <c r="E24" t="n">
-        <v>-13245378.91382747</v>
+        <v>7825801.35194401</v>
       </c>
       <c r="F24" t="n">
-        <v>-101391599.8624936</v>
+        <v>-99917231.9799964</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>-101391599.8624936</v>
+        <v>-99917231.9799964</v>
       </c>
     </row>
     <row r="25">
@@ -1505,13 +1505,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1630303405.995301</v>
+        <v>1631183632.847675</v>
       </c>
       <c r="E27" t="n">
-        <v>416903410.0818864</v>
+        <v>413192224.0807344</v>
       </c>
       <c r="F27" t="n">
-        <v>2047206816.077187</v>
+        <v>2044375856.92841</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>2047206816.077187</v>
+        <v>2044375856.92841</v>
       </c>
     </row>
     <row r="28">
@@ -1539,13 +1539,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>4076747099.872595</v>
+        <v>4079284878.85129</v>
       </c>
       <c r="E28" t="n">
-        <v>1214999554.923893</v>
+        <v>1213216973.734823</v>
       </c>
       <c r="F28" t="n">
-        <v>5291746654.796488</v>
+        <v>5292501852.586112</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>5291746654.796488</v>
+        <v>5292501852.586112</v>
       </c>
     </row>
     <row r="29">
@@ -1607,13 +1607,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>-2040109369.00206</v>
+        <v>-2069717398.896387</v>
       </c>
       <c r="E30" t="n">
-        <v>-17827496.49511871</v>
+        <v>-18562065.64174477</v>
       </c>
       <c r="F30" t="n">
-        <v>-2057936865.497179</v>
+        <v>-2088279464.538132</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>-2057936865.497179</v>
+        <v>-2088279464.538132</v>
       </c>
     </row>
     <row r="31">
@@ -1641,13 +1641,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>-1727986719.141655</v>
+        <v>-1728327152.573152</v>
       </c>
       <c r="E31" t="n">
-        <v>-43990450.20683838</v>
+        <v>-43785740.17595147</v>
       </c>
       <c r="F31" t="n">
-        <v>-1771977169.348494</v>
+        <v>-1772112892.749104</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>-1771977169.348494</v>
+        <v>-1772112892.749104</v>
       </c>
     </row>
     <row r="32">
@@ -1675,13 +1675,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1505976976.942232</v>
+        <v>1583395833.267716</v>
       </c>
       <c r="E32" t="n">
-        <v>210260783.4968137</v>
+        <v>217355097.5827104</v>
       </c>
       <c r="F32" t="n">
-        <v>1716237760.439046</v>
+        <v>1800750930.850427</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>1716237760.439046</v>
+        <v>1800750930.850427</v>
       </c>
     </row>
     <row r="33">
@@ -1709,13 +1709,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>-91746843.35194483</v>
+        <v>-101691890.0460503</v>
       </c>
       <c r="E33" t="n">
-        <v>-9319613.642388146</v>
+        <v>3770108.42507934</v>
       </c>
       <c r="F33" t="n">
-        <v>-101066456.9943329</v>
+        <v>-97921781.62097092</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>-101066456.9943329</v>
+        <v>-97921781.62097092</v>
       </c>
     </row>
     <row r="34">
@@ -1811,13 +1811,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1718070353.025799</v>
+        <v>1719318005.3373</v>
       </c>
       <c r="E36" t="n">
-        <v>430613497.4205008</v>
+        <v>426812475.1325808</v>
       </c>
       <c r="F36" t="n">
-        <v>2148683850.4463</v>
+        <v>2146130480.469881</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>2148683850.4463</v>
+        <v>2146130480.469881</v>
       </c>
     </row>
     <row r="37">
@@ -1845,13 +1845,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4367865837.054114</v>
+        <v>4369321729.236615</v>
       </c>
       <c r="E37" t="n">
-        <v>915899295.0771817</v>
+        <v>915290010.7673179</v>
       </c>
       <c r="F37" t="n">
-        <v>5283765132.131296</v>
+        <v>5284611740.003933</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>5283765132.131296</v>
+        <v>5284611740.003933</v>
       </c>
     </row>
     <row r="38">
@@ -1913,13 +1913,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>-2035829947.451668</v>
+        <v>-2065261814.569718</v>
       </c>
       <c r="E39" t="n">
-        <v>-17776971.56842878</v>
+        <v>-18509490.79661817</v>
       </c>
       <c r="F39" t="n">
-        <v>-2053606919.020097</v>
+        <v>-2083771305.366336</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>-2053606919.020097</v>
+        <v>-2083771305.366336</v>
       </c>
     </row>
     <row r="40">
@@ -1947,13 +1947,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>-1706567718.532032</v>
+        <v>-1706947892.201009</v>
       </c>
       <c r="E40" t="n">
-        <v>-56761800.53062917</v>
+        <v>-56557264.6895509</v>
       </c>
       <c r="F40" t="n">
-        <v>-1763329519.062661</v>
+        <v>-1763505156.89056</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>-1763329519.062661</v>
+        <v>-1763505156.89056</v>
       </c>
     </row>
     <row r="41">
@@ -1981,13 +1981,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1464911848.915145</v>
+        <v>1544181776.842392</v>
       </c>
       <c r="E41" t="n">
-        <v>206105624.0048289</v>
+        <v>213394328.8999861</v>
       </c>
       <c r="F41" t="n">
-        <v>1671017472.919974</v>
+        <v>1757576105.742378</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1671017472.919974</v>
+        <v>1757576105.742378</v>
       </c>
     </row>
     <row r="42">
@@ -2015,13 +2015,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>-89260975.01371798</v>
+        <v>-103123117.5636715</v>
       </c>
       <c r="E42" t="n">
-        <v>-11477510.98777739</v>
+        <v>5832949.61622251</v>
       </c>
       <c r="F42" t="n">
-        <v>-100738486.0014953</v>
+        <v>-97290167.947449</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>-100738486.0014953</v>
+        <v>-97290167.947449</v>
       </c>
     </row>
     <row r="43">
@@ -2117,13 +2117,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1667639460.942172</v>
+        <v>1668722714.579239</v>
       </c>
       <c r="E45" t="n">
-        <v>421374669.2835167</v>
+        <v>417642140.1525146</v>
       </c>
       <c r="F45" t="n">
-        <v>2089014130.225689</v>
+        <v>2086364854.731754</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>2089014130.225689</v>
+        <v>2086364854.731754</v>
       </c>
     </row>
     <row r="46">
@@ -2151,13 +2151,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4209706772.111761</v>
+        <v>4211643458.974069</v>
       </c>
       <c r="E46" t="n">
-        <v>1052638446.31821</v>
+        <v>1051689241.133928</v>
       </c>
       <c r="F46" t="n">
-        <v>5262345218.429971</v>
+        <v>5263332700.107997</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>5262345218.429971</v>
+        <v>5263332700.107997</v>
       </c>
     </row>
     <row r="47">
@@ -2219,13 +2219,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>-2062058668.263331</v>
+        <v>-2092575779.136144</v>
       </c>
       <c r="E48" t="n">
-        <v>-18069356.33798468</v>
+        <v>-18813949.17801103</v>
       </c>
       <c r="F48" t="n">
-        <v>-2080128024.601315</v>
+        <v>-2111389728.314155</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>-2080128024.601315</v>
+        <v>-2111389728.314155</v>
       </c>
     </row>
     <row r="49">
@@ -2253,13 +2253,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>-1728904985.836331</v>
+        <v>-1728936081.371238</v>
       </c>
       <c r="E49" t="n">
-        <v>-44012024.86888601</v>
+        <v>-43805955.95861973</v>
       </c>
       <c r="F49" t="n">
-        <v>-1772917010.705217</v>
+        <v>-1772742037.329858</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>-1772917010.705217</v>
+        <v>-1772742037.329858</v>
       </c>
     </row>
     <row r="50">
@@ -2287,13 +2287,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1479015826.853442</v>
+        <v>1562586713.913684</v>
       </c>
       <c r="E50" t="n">
-        <v>209484658.562648</v>
+        <v>216998146.7390104</v>
       </c>
       <c r="F50" t="n">
-        <v>1688500485.41609</v>
+        <v>1779584860.652695</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>1688500485.41609</v>
+        <v>1779584860.652695</v>
       </c>
     </row>
     <row r="51">
@@ -2321,13 +2321,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>-91152904.78500237</v>
+        <v>-106395541.5802239</v>
       </c>
       <c r="E51" t="n">
-        <v>-10701706.44809381</v>
+        <v>5509528.18466062</v>
       </c>
       <c r="F51" t="n">
-        <v>-101854611.2330962</v>
+        <v>-100886013.3955633</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2335,7 +2335,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>-101854611.2330962</v>
+        <v>-100886013.3955633</v>
       </c>
     </row>
     <row r="52">
@@ -2423,13 +2423,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1689551241.756139</v>
+        <v>1690612874.487984</v>
       </c>
       <c r="E54" t="n">
-        <v>428046921.0083535</v>
+        <v>424251848.6959267</v>
       </c>
       <c r="F54" t="n">
-        <v>2117598162.764492</v>
+        <v>2114864723.183911</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>2117598162.764492</v>
+        <v>2114864723.183911</v>
       </c>
     </row>
     <row r="55">
@@ -2457,13 +2457,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>4258672231.387065</v>
+        <v>4260673619.573924</v>
       </c>
       <c r="E55" t="n">
-        <v>1060871481.666171</v>
+        <v>1059437047.426642</v>
       </c>
       <c r="F55" t="n">
-        <v>5319543713.053237</v>
+        <v>5320110667.000566</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2471,7 +2471,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>5319543713.053237</v>
+        <v>5320110667.000566</v>
       </c>
     </row>
     <row r="56">
@@ -2525,13 +2525,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>-2054147066.18232</v>
+        <v>-2084335943.332529</v>
       </c>
       <c r="E57" t="n">
-        <v>-17983662.59355108</v>
+        <v>-18724684.28090506</v>
       </c>
       <c r="F57" t="n">
-        <v>-2072130728.775872</v>
+        <v>-2103060627.613434</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>-2072130728.775872</v>
+        <v>-2103060627.613434</v>
       </c>
     </row>
     <row r="58">
@@ -2559,13 +2559,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>-1738070634.351016</v>
+        <v>-1738222343.200953</v>
       </c>
       <c r="E58" t="n">
-        <v>-38293460.94437269</v>
+        <v>-38087921.63274255</v>
       </c>
       <c r="F58" t="n">
-        <v>-1776364095.295389</v>
+        <v>-1776310264.833696</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>-1776364095.295389</v>
+        <v>-1776310264.833696</v>
       </c>
     </row>
     <row r="59">
@@ -2593,13 +2593,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1509299454.73327</v>
+        <v>1589304929.729342</v>
       </c>
       <c r="E59" t="n">
-        <v>211683870.2150885</v>
+        <v>218924067.8768276</v>
       </c>
       <c r="F59" t="n">
-        <v>1720983324.948359</v>
+        <v>1808228997.60617</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>1720983324.948359</v>
+        <v>1808228997.60617</v>
       </c>
     </row>
     <row r="60">
@@ -2627,13 +2627,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>-92528512.11000258</v>
+        <v>-103671322.0597626</v>
       </c>
       <c r="E60" t="n">
-        <v>-9119557.675629426</v>
+        <v>3830635.129368225</v>
       </c>
       <c r="F60" t="n">
-        <v>-101648069.785632</v>
+        <v>-99840686.93039435</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2641,7 +2641,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>-101648069.785632</v>
+        <v>-99840686.93039435</v>
       </c>
     </row>
     <row r="61">
@@ -2729,13 +2729,13 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1724635591.07882</v>
+        <v>1725852550.461277</v>
       </c>
       <c r="E63" t="n">
-        <v>433301083.4391299</v>
+        <v>429472849.6781961</v>
       </c>
       <c r="F63" t="n">
-        <v>2157936674.51795</v>
+        <v>2155325400.139473</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2743,7 +2743,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>2157936674.51795</v>
+        <v>2155325400.139473</v>
       </c>
     </row>
     <row r="64">
@@ -2763,13 +2763,13 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>4377306022.247397</v>
+        <v>4378850688.133968</v>
       </c>
       <c r="E64" t="n">
-        <v>935656590.6933227</v>
+        <v>934741399.0990008</v>
       </c>
       <c r="F64" t="n">
-        <v>5312962612.94072</v>
+        <v>5313592087.232969</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2777,7 +2777,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>5312962612.94072</v>
+        <v>5313592087.232969</v>
       </c>
     </row>
   </sheetData>
@@ -2848,13 +2848,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-11499397.94553286</v>
+        <v>24519781.54135217</v>
       </c>
       <c r="C2" t="n">
-        <v>1805733237.543785</v>
+        <v>1833105266.858336</v>
       </c>
       <c r="D2" t="n">
-        <v>1794233839.598252</v>
+        <v>1857625048.399688</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -2862,16 +2862,16 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-122122221.6511104</v>
+        <v>-117121148.4077153</v>
       </c>
       <c r="G2" t="n">
-        <v>-10.1768518042592</v>
+        <v>-9.760095700642943</v>
       </c>
       <c r="H2" t="n">
-        <v>-122122221.6511104</v>
+        <v>-117121148.4077153</v>
       </c>
       <c r="I2" t="n">
-        <v>-10.1768518042592</v>
+        <v>-9.760095700642943</v>
       </c>
     </row>
     <row r="3">
@@ -2881,13 +2881,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>644826416.1403605</v>
+        <v>688555439.7483164</v>
       </c>
       <c r="C3" t="n">
-        <v>1405066494.163117</v>
+        <v>1414007362.965398</v>
       </c>
       <c r="D3" t="n">
-        <v>2049892910.303477</v>
+        <v>2102562802.713715</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -2895,16 +2895,16 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>133536849.0541148</v>
+        <v>127816605.906311</v>
       </c>
       <c r="G3" t="n">
-        <v>11.12807075450957</v>
+        <v>10.65138382552592</v>
       </c>
       <c r="H3" t="n">
-        <v>66768424.52705741</v>
+        <v>63908302.95315552</v>
       </c>
       <c r="I3" t="n">
-        <v>5.564035377254784</v>
+        <v>5.32569191276296</v>
       </c>
     </row>
     <row r="4">
@@ -2914,13 +2914,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>128267619.9428985</v>
+        <v>167096018.2578724</v>
       </c>
       <c r="C4" t="n">
-        <v>1741991483.446984</v>
+        <v>1764753415.730354</v>
       </c>
       <c r="D4" t="n">
-        <v>1870259103.389882</v>
+        <v>1931849433.988226</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -2928,16 +2928,16 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-46096957.85948014</v>
+        <v>-42896762.81917739</v>
       </c>
       <c r="G4" t="n">
-        <v>-3.841413154956678</v>
+        <v>-3.574730234931449</v>
       </c>
       <c r="H4" t="n">
-        <v>-46096957.85948014</v>
+        <v>-42896762.81917739</v>
       </c>
       <c r="I4" t="n">
-        <v>-3.841413154956678</v>
+        <v>-3.574730234931449</v>
       </c>
     </row>
     <row r="5">
@@ -2947,13 +2947,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>441211255.9515758</v>
+        <v>481440146.7511313</v>
       </c>
       <c r="C5" t="n">
-        <v>1510390903.507896</v>
+        <v>1525634773.947738</v>
       </c>
       <c r="D5" t="n">
-        <v>1951602159.459472</v>
+        <v>2007074920.698869</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -2961,16 +2961,16 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>35246098.21010947</v>
+        <v>32328723.89146566</v>
       </c>
       <c r="G5" t="n">
-        <v>2.937174850842456</v>
+        <v>2.694060324288805</v>
       </c>
       <c r="H5" t="n">
-        <v>17623049.10505474</v>
+        <v>16164361.94573283</v>
       </c>
       <c r="I5" t="n">
-        <v>1.468587425421228</v>
+        <v>1.347030162144403</v>
       </c>
     </row>
     <row r="6">
@@ -2980,13 +2980,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>290435878.7641941</v>
+        <v>329051563.8538368</v>
       </c>
       <c r="C6" t="n">
-        <v>1605422703.504003</v>
+        <v>1624812151.300765</v>
       </c>
       <c r="D6" t="n">
-        <v>1895858582.268197</v>
+        <v>1953863715.154602</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -2994,16 +2994,16 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>-20497478.98116589</v>
+        <v>-20882481.65280151</v>
       </c>
       <c r="G6" t="n">
-        <v>-1.70812324843049</v>
+        <v>-1.740206804400126</v>
       </c>
       <c r="H6" t="n">
-        <v>-20497478.98116589</v>
+        <v>-20882481.65280151</v>
       </c>
       <c r="I6" t="n">
-        <v>-1.70812324843049</v>
+        <v>-1.740206804400126</v>
       </c>
     </row>
     <row r="7">
@@ -3013,13 +3013,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>298928954.0276618</v>
+        <v>339772018.8036674</v>
       </c>
       <c r="C7" t="n">
-        <v>1638294398.295353</v>
+        <v>1656251090.622754</v>
       </c>
       <c r="D7" t="n">
-        <v>1937223352.323015</v>
+        <v>1996023109.426422</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -3027,16 +3027,16 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>20867291.07365227</v>
+        <v>21276912.61901784</v>
       </c>
       <c r="G7" t="n">
-        <v>1.738940922804356</v>
+        <v>1.77307605158482</v>
       </c>
       <c r="H7" t="n">
-        <v>10433645.53682613</v>
+        <v>10638456.30950892</v>
       </c>
       <c r="I7" t="n">
-        <v>0.8694704614021779</v>
+        <v>0.8865380257924099</v>
       </c>
     </row>
     <row r="8">
@@ -3046,13 +3046,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>429051275.6851131</v>
+        <v>470334980.0003086</v>
       </c>
       <c r="C8" t="n">
-        <v>1539327935.588841</v>
+        <v>1554239418.324598</v>
       </c>
       <c r="D8" t="n">
-        <v>1968379211.273955</v>
+        <v>2024574398.324907</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -3060,16 +3060,16 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>52023150.02459216</v>
+        <v>49828201.51750278</v>
       </c>
       <c r="G8" t="n">
-        <v>4.335262502049346</v>
+        <v>4.152350126458566</v>
       </c>
       <c r="H8" t="n">
-        <v>26011575.01229608</v>
+        <v>24914100.75875139</v>
       </c>
       <c r="I8" t="n">
-        <v>2.167631251024673</v>
+        <v>2.076175063229283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>